<commit_message>
Treat DateTimeOffset as text and update docs
Excel cannot represent timezone offsets in numeric date cells, so DateTimeOffset values are written as formatted strings to preserve the offset and no NumberFormat is applied. Update Renderer.cs to stop assigning style.NumberFormat and write the formatted string via ToString(format, Culture). Clarify behavior in the README (noting Excel will treat such cells as plain text for sorting/filtering/arithmetic and the format is applied at write time). Update verified test XLSX accordingly.
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/DateFormats.Test.verified.xlsx
+++ b/src/Excelsior.Tests/DateFormats.Test.verified.xlsx
@@ -9,10 +9,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-MM-dd"/>
     <numFmt numFmtId="165" formatCode="yyyy-MM-dd HH:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="yyyy-MM-dd HH:mm:ss z"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -51,7 +50,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="0" applyFill="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="0" applyFill="0" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>

</xml_diff>